<commit_message>
more wind files now that there is a short burn in period
</commit_message>
<xml_diff>
--- a/scenarios/v06/actions_1.xlsx
+++ b/scenarios/v06/actions_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\scenarios\v06\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\UNIMELB\outbreaksimulator\scenarios\v06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6945473A-A6C3-4D17-83F7-490DE73E8498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC66AD6-ECBE-4D72-8635-1807F8BA2CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31455" yWindow="1530" windowWidth="25005" windowHeight="12570" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
   </bookViews>
   <sheets>
     <sheet name="jobs" sheetId="1" r:id="rId1"/>
@@ -492,10 +492,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>68</v>
+        <v>171</v>
       </c>
       <c r="B2" s="1">
-        <v>46055</v>
+        <v>46039</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -503,10 +503,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>68</v>
+        <v>171</v>
       </c>
       <c r="B3" s="1">
-        <v>46055</v>
+        <v>46039</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>68</v>
+        <v>171</v>
       </c>
       <c r="B4" s="1">
-        <v>46056</v>
+        <v>46040</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
@@ -551,7 +551,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>68</v>
+        <v>171</v>
       </c>
       <c r="B2">
         <v>1</v>

</xml_diff>

<commit_message>
adding in new surveillence options (partial implementation)
</commit_message>
<xml_diff>
--- a/scenarios/v06/actions_1.xlsx
+++ b/scenarios/v06/actions_1.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\UNIMELB\outbreaksimulator\scenarios\v06\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\scenarios\v06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC66AD6-ECBE-4D72-8635-1807F8BA2CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02932A8-D750-4F20-A1AF-8D5F45D44E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
+    <workbookView xWindow="30675" yWindow="1860" windowWidth="24030" windowHeight="12960" activeTab="1" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
   </bookViews>
   <sheets>
     <sheet name="jobs" sheetId="1" r:id="rId1"/>
-    <sheet name="zones" sheetId="3" r:id="rId2"/>
-    <sheet name="notes" sheetId="2" r:id="rId3"/>
+    <sheet name="zone_jobs" sheetId="4" r:id="rId2"/>
+    <sheet name="zones" sheetId="3" r:id="rId3"/>
+    <sheet name="notes" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
   <si>
     <t>ID</t>
   </si>
@@ -49,42 +50,12 @@
     <t>date_scheduled</t>
   </si>
   <si>
-    <t>actions that can be done</t>
-  </si>
-  <si>
-    <t>extra details?</t>
-  </si>
-  <si>
-    <t>clinical inspection</t>
-  </si>
-  <si>
-    <t>lab test</t>
-  </si>
-  <si>
-    <t>culling</t>
-  </si>
-  <si>
-    <t>the number of animals culled on the scheduled date</t>
-  </si>
-  <si>
-    <t>vaccination</t>
-  </si>
-  <si>
-    <t>the number of animals vaccinated on the scheduled date</t>
-  </si>
-  <si>
-    <t>decontamination?</t>
-  </si>
-  <si>
     <t>radius_km</t>
   </si>
   <si>
     <t>zone_type</t>
   </si>
   <si>
-    <t>contact tracing</t>
-  </si>
-  <si>
     <t>RA</t>
   </si>
   <si>
@@ -98,15 +69,211 @@
   </si>
   <si>
     <t>ContactTracing</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>Cull</t>
+  </si>
+  <si>
+    <t>Vaccination</t>
+  </si>
+  <si>
+    <t>Jobs tab</t>
+  </si>
+  <si>
+    <t>specific_action</t>
+  </si>
+  <si>
+    <t>detection_prob</t>
+  </si>
+  <si>
+    <t>Surveillance</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>property ID (sim_id)</t>
+  </si>
+  <si>
+    <t>circular radius around property (in km)</t>
+  </si>
+  <si>
+    <t>Free text notes</t>
+  </si>
+  <si>
+    <t>Phone Surveillance</t>
+  </si>
+  <si>
+    <t>Field Surveillance</t>
+  </si>
+  <si>
+    <t>Self-reporting Surveillance</t>
+  </si>
+  <si>
+    <t>zone_name</t>
+  </si>
+  <si>
+    <t>Example rows</t>
+  </si>
+  <si>
+    <t>Date when action will complete</t>
+  </si>
+  <si>
+    <t>ClinicalObservation, ContactTracing, LabTesting, Cull, Vaccination, Surveillance</t>
+  </si>
+  <si>
+    <t>Used when action=Surveillance. Possible inputs: Field Surveillance, Phone Surveillance, Self-reporting Surveillance</t>
+  </si>
+  <si>
+    <t>ID*</t>
+  </si>
+  <si>
+    <t>date_scheduled*</t>
+  </si>
+  <si>
+    <t>action*</t>
+  </si>
+  <si>
+    <t>If action=Culled, then the number of animals culled on the scheduled date.
+If action=Vaccination, then the number of animals vaccinated on the scheduled date</t>
+  </si>
+  <si>
+    <t>Detail / possible values</t>
+  </si>
+  <si>
+    <t>Used when action=Surveillance. Detection probability of the specific surveillance. If not provided, then pre-coded values will be used.</t>
+  </si>
+  <si>
+    <t>Any notes for personal reference, not used by the simulation model</t>
+  </si>
+  <si>
+    <t>Corresponds to site visit to property with sim_id = 68 on the 12th Jan, conducting a clinical observation of chickens on site</t>
+  </si>
+  <si>
+    <t>Results of a PCR test on property 68 is received on the scheduled date (12 Jan)</t>
+  </si>
+  <si>
+    <t>35k chickens are culled on property 80 on the 13th Jan</t>
+  </si>
+  <si>
+    <t>Action type</t>
+  </si>
+  <si>
+    <t>Implemented action/information obtained</t>
+  </si>
+  <si>
+    <t>Site visit by vet. Obtains property information (number of sheds, number of animals etc) and if there are any clinical signs</t>
+  </si>
+  <si>
+    <t>Conducts forward and backward contact tracing</t>
+  </si>
+  <si>
+    <t>Conducts a high sensitivity PCR test</t>
+  </si>
+  <si>
+    <t>Culls chickens and destroys any eggs. Automatic disposal and decontamination after culling.</t>
+  </si>
+  <si>
+    <t>Not implemented</t>
+  </si>
+  <si>
+    <t>Various additional surveillence methods. All methods obtain property information (number of sheds, number of animals etc) and if there are any clinical signs. Success of clinical sign identification/reporting varies by specific surveillence type / input detection_prob parameter</t>
+  </si>
+  <si>
+    <t>Zone_Jobs tab</t>
+  </si>
+  <si>
+    <t>zone_parameter</t>
+  </si>
+  <si>
+    <t>Enhanced Passive Surveillence</t>
+  </si>
+  <si>
+    <t>Population-level Surveillance</t>
+  </si>
+  <si>
+    <t>Wild Animal Surveillence</t>
+  </si>
+  <si>
+    <t>Environmental Surveillence</t>
+  </si>
+  <si>
+    <t>radius_km*</t>
+  </si>
+  <si>
+    <t>zone_type*</t>
+  </si>
+  <si>
+    <t>zone_name*</t>
+  </si>
+  <si>
+    <t>Radius around property ID where action will take place</t>
+  </si>
+  <si>
+    <t>Actions possible: Enhanced Passive Surveillence, Population-level Surveillance, Wild Animal Surveillence, Environmental Surveillence</t>
+  </si>
+  <si>
+    <t>Reference name for the zone action (given that we can't use the property ID)</t>
+  </si>
+  <si>
+    <t>A parameter to adjust the sensitivity of the action</t>
+  </si>
+  <si>
+    <t>RA, CA</t>
+  </si>
+  <si>
+    <t>Implementation</t>
+  </si>
+  <si>
+    <t>Reistricted area - no movements</t>
+  </si>
+  <si>
+    <t>Control area - reduced movements, for designating PORs</t>
+  </si>
+  <si>
+    <t>Increases self-reporting probability</t>
+  </si>
+  <si>
+    <t>eDNA testing within particular zone</t>
+  </si>
+  <si>
+    <t>mortality sampling of known premises within particular zone, assumes pooled PCR</t>
+  </si>
+  <si>
+    <t>mortality sampling of wild birds within particular zone, assumes pooled PCR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -120,7 +287,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -128,13 +295,257 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -469,14 +880,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EC4FC7D-172B-4FB5-8C5B-14F92FDF678B}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="18.125" customWidth="1"/>
+    <col min="4" max="4" width="22.125" customWidth="1"/>
+    <col min="5" max="5" width="14.875" customWidth="1"/>
+    <col min="7" max="7" width="20.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -487,41 +901,95 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>171</v>
       </c>
       <c r="B2" s="1">
-        <v>46039</v>
+        <v>46042</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>171</v>
       </c>
       <c r="B3" s="1">
-        <v>46039</v>
+        <v>46042</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>171</v>
       </c>
       <c r="B4" s="1">
-        <v>46040</v>
+        <v>46043</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
-      </c>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="1"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B17" s="1"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B18" s="1"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B19" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -529,36 +997,52 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB002FF-49E8-4F00-BBA1-9E981B1CFB66}">
-  <dimension ref="A1:C2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71766014-C2B2-4522-9F6F-9B568A56B108}">
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.375" customWidth="1"/>
-    <col min="3" max="3" width="13.125" customWidth="1"/>
-    <col min="4" max="4" width="17.375" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="29.875" customWidth="1"/>
+    <col min="5" max="5" width="16.875" customWidth="1"/>
+    <col min="6" max="6" width="14.75" customWidth="1"/>
+    <col min="7" max="7" width="21.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>171</v>
-      </c>
-      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -566,59 +1050,639 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA9FDAFF-FC45-49EA-B8F5-53ECA0B0E905}">
-  <dimension ref="A1:B7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB002FF-49E8-4F00-BBA1-9E981B1CFB66}">
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.25" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="2" max="2" width="11.375" customWidth="1"/>
+    <col min="3" max="3" width="23.875" customWidth="1"/>
+    <col min="4" max="4" width="17.375" customWidth="1"/>
+    <col min="5" max="5" width="13.875" customWidth="1"/>
+    <col min="6" max="6" width="18.375" customWidth="1"/>
+    <col min="7" max="7" width="21.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>171</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>171</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA9FDAFF-FC45-49EA-B8F5-53ECA0B0E905}">
+  <dimension ref="A1:H43"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.875" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18.875" customWidth="1"/>
+    <col min="4" max="4" width="22.125" customWidth="1"/>
+    <col min="5" max="5" width="16.375" customWidth="1"/>
+    <col min="6" max="6" width="17.75" customWidth="1"/>
+    <col min="7" max="7" width="64.125" customWidth="1"/>
+    <col min="8" max="8" width="25.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="19"/>
+      <c r="F2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="30"/>
+    </row>
+    <row r="3" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="27"/>
+      <c r="D3" s="28"/>
+      <c r="F3" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="32"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="28"/>
+      <c r="F4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="34"/>
+    </row>
+    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="21"/>
+      <c r="D5" s="22"/>
+      <c r="F5" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="H5" s="34"/>
+    </row>
+    <row r="6" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="21"/>
+      <c r="D6" s="22"/>
+      <c r="F6" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="32"/>
+    </row>
+    <row r="7" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="21"/>
+      <c r="D7" s="22"/>
+      <c r="F7" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" s="36"/>
+    </row>
+    <row r="8" spans="1:8" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="28"/>
+      <c r="F8" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="38"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="40"/>
+      <c r="D9" s="41"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A13" s="4">
+        <v>68</v>
+      </c>
+      <c r="B13" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="4">
+        <v>68</v>
+      </c>
+      <c r="B14" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="4">
+        <v>68</v>
+      </c>
+      <c r="B15" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="4">
+        <v>80</v>
+      </c>
+      <c r="B16" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4">
+        <v>35000</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="4">
+        <v>100</v>
+      </c>
+      <c r="B17" s="10">
+        <v>46036</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="4">
+        <v>101</v>
+      </c>
+      <c r="B18" s="10">
+        <v>46036</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="4">
+        <v>500</v>
+      </c>
+      <c r="B19" s="10">
+        <v>46036</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="22" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A23" s="14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="F24" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G24" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="H24" s="30"/>
+    </row>
+    <row r="25" spans="1:8" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="21"/>
+      <c r="D25" s="22"/>
+      <c r="F25" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="G25" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="H25" s="32"/>
+    </row>
+    <row r="26" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" s="21"/>
+      <c r="D26" s="22"/>
+      <c r="F26" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G26" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="H26" s="34"/>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="21"/>
+      <c r="D27" s="22"/>
+      <c r="F27" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G27" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="H27" s="34"/>
+    </row>
+    <row r="28" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="21"/>
+      <c r="D28" s="22"/>
+      <c r="F28" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G28" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="H28" s="32"/>
+    </row>
+    <row r="29" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="21"/>
+      <c r="D29" s="22"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="36"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="21"/>
+      <c r="D30" s="22"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="37"/>
+      <c r="H30" s="38"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="24"/>
+      <c r="D31" s="25"/>
+    </row>
+    <row r="33" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A33" s="14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="18"/>
+      <c r="D34" s="19"/>
+      <c r="F34" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G34" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="H34" s="30"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="21"/>
+      <c r="D35" s="22"/>
+      <c r="F35" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="G35" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="H35" s="32"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="21"/>
+      <c r="D36" s="22"/>
+      <c r="F36" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="H36" s="43"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" s="21"/>
+      <c r="D37" s="22"/>
+    </row>
+    <row r="38" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="C38" s="24"/>
+      <c r="D38" s="25"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="16"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="21"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="16"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" s="16"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+    </row>
+    <row r="42" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+    </row>
+    <row r="43" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="41">
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B31:D31"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>